<commit_message>
Complete large-account list to 500
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9KJnaVmdH42r75H4m1WYx
</commit_message>
<xml_diff>
--- a/prospection/grands-comptes-PIWA.xlsx
+++ b/prospection/grands-comptes-PIWA.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Grands comptes'!$A$1:$P$499</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Grands comptes'!$A$1:$P$500</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P499"/>
+  <dimension ref="A1:P500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -41375,10 +41375,92 @@
       <c r="O499" s="2" t="inlineStr"/>
       <c r="P499" s="2" t="inlineStr"/>
     </row>
+    <row r="500" ht="120" customHeight="1">
+      <c r="A500" s="2" t="n">
+        <v>499</v>
+      </c>
+      <c r="B500" s="2" t="inlineStr">
+        <is>
+          <t>Hachette Livre</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>Édition</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>Vanves</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="inlineStr">
+        <is>
+          <t>à vérifier</t>
+        </is>
+      </c>
+      <c r="F500" s="2" t="inlineStr">
+        <is>
+          <t>Grand groupe</t>
+        </is>
+      </c>
+      <c r="G500" s="2" t="inlineStr">
+        <is>
+          <t>Vidéos de lancement produit et vidéos de marque employeur.</t>
+        </is>
+      </c>
+      <c r="H500" s="2" t="inlineStr">
+        <is>
+          <t>PDG / Directeur général ; à défaut Directeur de la communication ou DRH</t>
+        </is>
+      </c>
+      <c r="I500" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn (chercher « PDG Hachette Livre ») ; courrier au siège ; formulaire de contact du site</t>
+        </is>
+      </c>
+      <c r="J500" s="2" t="inlineStr">
+        <is>
+          <t>Une vidéo d'exception pour Hachette Livre, pour un budget maîtrisé</t>
+        </is>
+      </c>
+      <c r="K500" s="2" t="inlineStr">
+        <is>
+          <t>Madame, Monsieur le Président,
+Je me permets de m'adresser directement à vous. PIWA Studio est le studio vidéo du groupe MONTAUGEM, société au capital de 5 177 000 €. Nos équipes conçoivent des vidéos motion design haut de gamme pour les entreprises : script, voix off, musique originale et animation, dans plus de 25 langues.
+Pour Hachette Livre, une première idée : vidéos de lancement produit et vidéos de marque employeur.
+Notre proposition est simple : une vidéo d'un niveau agence, livrée en 7 jours, pour un budget très maîtrisé, à partir de 990 € HT. Une première vidéo permet à vos équipes de juger sur pièce, sans engagement de volume.
+Quelques réalisations : https://dgjmfrbv4k-lab.github.io/NOXEM-GROUP/piwa/?v=2#nointro
+Je serais honoré de pouvoir échanger quelques minutes avec vous ou avec la personne de votre choix (communication, marketing ou ressources humaines).
+Je vous prie d'agréer, Madame, Monsieur le Président, l'expression de mes salutations distinguées.
+Kevin
+PIWA Studio, groupe MONTAUGEM (capital de 5 177 000 €)
++33 6 86 12 13 71 (appel ou WhatsApp)
+Si vous ne souhaitez plus être contacté, répondez simplement STOP.</t>
+        </is>
+      </c>
+      <c r="L500" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour, Kevin de PIWA Studio, studio vidéo du groupe MONTAUGEM (capital de 5 177 000 €). Nos équipes réalisent des vidéos motion design haut de gamme livrées en 7 jours, à partir de 990 € HT. Je serais ravi d'en proposer une pour Hachette Livre. Nos réalisations : https://dgjmfrbv4k-lab.github.io/NOXEM-GROUP/piwa/?v=2#nointro</t>
+        </is>
+      </c>
+      <c r="M500" s="2" t="inlineStr">
+        <is>
+          <t>À vérifier</t>
+        </is>
+      </c>
+      <c r="N500" s="2" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="O500" s="2" t="inlineStr"/>
+      <c r="P500" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P499"/>
+  <autoFilter ref="A1:P500"/>
   <dataValidations count="1">
-    <dataValidation sqref="N2:N499" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"À contacter,Envoyé,Relancé,Répondu,RDV,Devis envoyé,Signé,Pas intéressé"</formula1>
     </dataValidation>
   </dataValidations>
@@ -41401,7 +41483,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>498 grandes entreprises, message adressé au PDG</t>
+          <t>499 grandes entreprises, message adressé au PDG</t>
         </is>
       </c>
     </row>

</xml_diff>